<commit_message>
feat: estandarización de codificación humana y matriz comparativa final v5
</commit_message>
<xml_diff>
--- a/Analisis_Cualitativo_MC_Limpio.xlsx
+++ b/Analisis_Cualitativo_MC_Limpio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\MEGADAPT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D53D978-91B6-4D58-90CF-801280CFC067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F52CCEFD-CBEC-4BF7-927C-1BB4203057ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79,8 +79,9 @@
     <t>ninguno</t>
   </si>
   <si>
-    <t>- Recomendar y dar seguimiento a las quejas ciudadanas.
-- Concluir el trámite de conciliación entre la autoridad y los ciudadanos.</t>
+    <t>Recomedar y dar segumiento 
+quejas ciudadanas. 
+Concluir en el tramite de consiliación entre la autoridad y  ciudadanos.</t>
   </si>
   <si>
     <t>Quejas por cobro y tarifas públicas  del agua. 
@@ -134,7 +135,7 @@
 </t>
   </si>
   <si>
-    <t>Capital está moviendo urbanización</t>
+    <t>- El capital está impulsando la urbanización.</t>
   </si>
   <si>
     <t xml:space="preserve">Desarrollo sector inmobiliario (SEDUVI y SOBSE)
@@ -235,12 +236,11 @@
     <t xml:space="preserve">Asentamientos humanos formales e informales </t>
   </si>
   <si>
-    <t xml:space="preserve">Cambio de  uso de suelo 
-Rescatar las barrancas
-Falta de infiltración
-Mala calidad 
-Tandeo
-</t>
+    <t>- Cambio de uso de suelo
+- Rescatar las barrancas
+- Falta de infiltración
+- Mala calidad
+- Tandeo</t>
   </si>
   <si>
     <t>Crecimiento urbano 
@@ -304,10 +304,10 @@
 Calidad</t>
   </si>
   <si>
-    <t>Inundaciones
-Escasez 
-Disponibilidad
-Distribución (tandeo)</t>
+    <t>- Inundaciones
+- Escasez
+- Disponibilidad
+- Distribución (tandeo)</t>
   </si>
   <si>
     <t>Lluvias

</xml_diff>